<commit_message>
Data update 2026-03-12: refresh ETL + GA load eval (fitness 4.1168)
data-only pipeline run: ETL fetched latest prices through 2026-03-10.
Features: 24352 → 15123 cols (62.1% kept), 134 tickers, 6727 rows.
GA load eval: win_rate=0.565, MDD=-24.0%, beat B&H 52.6% vs 6.5%, ALL PASS.
Top signals: PETR4 (98.6), AGRO3 (97.4), CXSE3 (88.1), CMIG4 (85.9).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/summary_latest.xlsx
+++ b/summary_latest.xlsx
@@ -2035,13 +2035,13 @@
         <v>54</v>
       </c>
       <c r="B48">
-        <v>2.058654706060585</v>
+        <v>2.067125694786445</v>
       </c>
       <c r="C48">
         <v>-0.2821828625695959</v>
       </c>
       <c r="D48">
-        <v>0.5299053957017699</v>
+        <v>0.5310129656503795</v>
       </c>
       <c r="E48">
         <v>150</v>
@@ -2050,7 +2050,7 @@
         <v>0.5866666666666667</v>
       </c>
       <c r="G48">
-        <v>0.008375598920036064</v>
+        <v>0.008394477613442509</v>
       </c>
       <c r="H48">
         <v>-0.4374445876444425</v>
@@ -15204,7 +15204,7 @@
         <v>109</v>
       </c>
       <c r="E347">
-        <v>43.1</v>
+        <v>43.3</v>
       </c>
       <c r="F347">
         <v>63.8</v>
@@ -19589,7 +19589,7 @@
         <v>0.1038</v>
       </c>
       <c r="E71">
-        <v>1.0685</v>
+        <v>1.0684</v>
       </c>
       <c r="F71">
         <v>91</v>
@@ -21489,7 +21489,7 @@
         <v>0.13</v>
       </c>
       <c r="E166">
-        <v>0.8434</v>
+        <v>0.8431</v>
       </c>
       <c r="F166">
         <v>78.2</v>
@@ -29369,10 +29369,10 @@
         <v>0.1993</v>
       </c>
       <c r="E560">
-        <v>0.8596</v>
+        <v>0.86</v>
       </c>
       <c r="F560">
-        <v>69.09999999999999</v>
+        <v>69.3</v>
       </c>
     </row>
     <row r="561" spans="1:6">
@@ -31629,7 +31629,7 @@
         <v>0.009900000000000001</v>
       </c>
       <c r="E673">
-        <v>0.8825</v>
+        <v>0.8826000000000001</v>
       </c>
       <c r="F673">
         <v>76.3</v>
@@ -34669,7 +34669,7 @@
         <v>0.1114</v>
       </c>
       <c r="E825">
-        <v>0.9644</v>
+        <v>0.9645</v>
       </c>
       <c r="F825">
         <v>82.3</v>
@@ -40789,7 +40789,7 @@
         <v>0.07820000000000001</v>
       </c>
       <c r="E1131">
-        <v>0.8909</v>
+        <v>0.8908</v>
       </c>
       <c r="F1131">
         <v>81.8</v>

</xml_diff>

<commit_message>
Fix timing/condicao consistency: integrated logic
Before: timing and condicao were independent (timing=no time but
condicao=Aguardar — contradictory). Now they are integrated:

- no time + above pivot → "COMPRAR: acima do Pivot, limite em X"
- no time + below pivot → "COMPRAR no rompimento de X, limite em Y"
- cedo + above pivot → "COMPRAR com cautela"
- cedo + below pivot → "AGUARDAR: comprar apenas se romper X"
- atrasado → "CAUTELA: considerar parcial"
- hold + muito cedo → "base em formacao"
- hold + cedo → "aguardar Stage 2"

https://claude.ai/code/session_012uaj5aSEsJzsdD3tyDK1oP
</commit_message>
<xml_diff>
--- a/summary_latest.xlsx
+++ b/summary_latest.xlsx
@@ -682,367 +682,367 @@
     <t>muito cedo</t>
   </si>
   <si>
-    <t>neutro</t>
+    <t>COMPRAR no rompimento de 63.76, limite em 61.80</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (63.76)</t>
+    <t>COMPRAR no rompimento de 51.16, limite em 50.20</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (51.16)</t>
+    <t>COMPRAR: acima do Pivot (65.27), limite em 64.32</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (65.27)</t>
+    <t>COMPRAR no rompimento de 57.25, limite em 56.08</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (57.25)</t>
+    <t>COMPRAR: acima do Pivot (29.17), limite em 28.94</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (29.17)</t>
+    <t>COMPRAR no rompimento de 47.32, limite em 46.47</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (47.32)</t>
+    <t>COMPRAR no rompimento de 33.35, limite em 33.17</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (33.35)</t>
+    <t>COMPRAR no rompimento de 20.27, limite em 19.38</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (20.27)</t>
+    <t>COMPRAR: acima do Pivot (48.21), limite em 46.85</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (48.21)</t>
+    <t>CAUTELA: atrasado, considerar parcial. Pivot em 9.43</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (9.43)</t>
+    <t>COMPRAR no rompimento de 18.37, limite em 18.12</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (18.37)</t>
+    <t>COMPRAR no rompimento de 157.47, limite em 154.14</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (157.47)</t>
+    <t>AGUARDAR: cedo, comprar apenas se romper 9.45</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (9.45)</t>
+    <t>COMPRAR no rompimento de 18.13, limite em 17.65</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (18.13)</t>
+    <t>COMPRAR: acima do Pivot (8.63), limite em 8.54</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (8.63)</t>
+    <t>COMPRAR: acima do Pivot (9.58), limite em 9.41</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (9.58)</t>
+    <t>COMPRAR no rompimento de 6.80, limite em 6.60</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (6.80)</t>
+    <t>AGUARDAR: cedo, comprar apenas se romper 21.05</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (21.05)</t>
+    <t>AGUARDAR: cedo, comprar apenas se romper 23.17</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (23.17)</t>
+    <t>COMPRAR: acima do Pivot (165.72), limite em 165.07</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (165.72)</t>
+    <t>AGUARDAR: cedo, comprar apenas se romper 8.88</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (8.88)</t>
+    <t>COMPRAR no rompimento de 29.07, limite em 28.42</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (29.07)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (114.65)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (114.65)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (23.53)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (23.53)</t>
+    <t>COMPRAR: acima do Pivot (45.02), limite em 44.45</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (45.02)</t>
+    <t>COMPRAR: acima do Pivot (28.43), limite em 27.93</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (28.43)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (46.77)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (46.77)</t>
+    <t>CAUTELA: atrasado, considerar parcial. Pivot em 16.41</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (16.41)</t>
+    <t>COMPRAR: acima do Pivot (94.66), limite em 94.20</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (94.66)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (31.27)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (31.27)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (57.83)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (57.83)</t>
+    <t>COMPRAR: acima do Pivot (14.20), limite em 14.00</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (14.20)</t>
+    <t>COMPRAR: acima do Pivot (20.35), limite em 20.34</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (20.35)</t>
+    <t>COMPRAR: acima do Pivot (103.53), limite em 103.16</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (103.53)</t>
+    <t>COMPRAR: acima do Pivot (32.55), limite em 32.06</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (32.55)</t>
+    <t>COMPRAR: acima do Pivot (52.82), limite em 51.91</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (52.82)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (16.02)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (16.02)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (8.80)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (8.80)</t>
+    <t>COMPRAR no rompimento de 10.32, limite em 10.27</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (10.32)</t>
+    <t>COMPRAR: acima do Pivot (19.65), limite em 19.37</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (19.65)</t>
+    <t>AGUARDAR: cedo, comprar apenas se romper 32.85</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (32.85)</t>
+    <t>COMPRAR: acima do Pivot (13.68), limite em 13.50</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (13.68)</t>
+    <t>COMPRAR no rompimento de 12.61, limite em 12.44</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (12.61)</t>
+    <t>COMPRAR: acima do Pivot (41.40), limite em 41.09</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (41.40)</t>
+    <t>AGUARDAR: cedo, comprar apenas se romper 48.78</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (48.78)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (108.80)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (108.80)</t>
+    <t>COMPRAR: limite em 4.62, stop em 4.51</t>
   </si>
   <si>
-    <t>Aguardar rompimento do Pivot (4.70)</t>
+    <t>COMPRAR: acima do Pivot (15.36), limite em 15.23</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (15.36)</t>
+    <t>COMPRAR com cautela: cedo mas acima do Pivot (25.94)</t>
   </si>
   <si>
-    <t>Comprar se abrir &gt; Pivot (25.94)</t>
+    <t>HOLD: abaixo do Pivot (9.68)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (9.68)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (0.09)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (0.09)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (6.79)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 6.79</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (52.09)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 52.09</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (52.15)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (52.15)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (14.20)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (14.35)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (2088.81)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 2126.69</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (9.05)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 9.05</t>
+    <t>HOLD: acima do Pivot (27.56) mas sem sinal</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 27.56</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (67403.34)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (68297.30)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (9.14)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 9.14</t>
+    <t>HOLD: acima do Pivot (36.70) mas sem sinal</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 36.70</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (6.38)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (6.48)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (31.13)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 31.72</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (96.91)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (98.45)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (93.10)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 93.10</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (4.95)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (5.00)</t>
+    <t>HOLD: abaixo do Pivot (43.21)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (43.21)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (108.39)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (108.39)</t>
+    <t>HOLD: acima do Pivot (35.11) mas sem sinal</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 35.11</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (1.25)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (1.29)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (381.16)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 382.40</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (14.24)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 14.24</t>
+    <t>HOLD: abaixo do Pivot (9.74)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (9.74)</t>
+    <t>HOLD: atrasado, evitar. Resistencia em R1 (21.50)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (21.24)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (141.03)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (141.03)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (13.42)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 13.57</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (53.79)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (54.23)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (4.27)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (4.33)</t>
+    <t>HOLD: acima do Pivot (35.29) mas sem sinal</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 35.29</t>
+    <t>HOLD: abaixo do Pivot (31.66)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (31.66)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (0.07)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (0.07)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (82.54)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 82.54</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (1.31)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 1.31</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (5.35)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 5.48</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (1.97)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 2.00</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (83.25)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (83.25)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (108.92)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (108.92)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (49.55)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (49.99)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (3.98)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 4.03</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (10.52)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (10.52)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (119.66)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (119.66)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (35.07)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 35.07</t>
+    <t>HOLD: acima do Pivot (59.54) mas sem sinal</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 59.54</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (6.20)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (6.27)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (17.65)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 17.65</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (75.79)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 76.53</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (40.84)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (40.84)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (23.06)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 23.26</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (19.70)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 19.70</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (82.37)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (84.24)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (99.74)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (100.25)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (0.51)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 0.52</t>
+    <t>HOLD: abaixo do Pivot (152.09)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (152.09)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (6.65)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 6.65</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (8.01)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 8.01</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (105.06)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 105.06</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (58.50)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 58.50</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (19.45)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 19.45</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (61.89)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (62.81)</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (8.94)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (8.94)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (64.57)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 64.78</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (155.76)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (155.94)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (14.95)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 15.15</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (98.69)</t>
   </si>
   <si>
-    <t>Abaixo do Pivot (98.94)</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (10.06)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 10.22</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (27.60)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 28.08</t>
+    <t>HOLD: cedo, aguardar Stage 2. Monitorar Pivot (43.95)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 43.95</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (91.22)</t>
   </si>
   <si>
-    <t>Aguardar confirmacao acima de 91.35</t>
-  </si>
-  <si>
-    <t>Aguardar confirmacao acima de 17.68</t>
+    <t>HOLD: muito cedo, base em formacao. Suporte em S1 (17.54)</t>
   </si>
   <si>
     <t>favoravel</t>
+  </si>
+  <si>
+    <t>neutro</t>
   </si>
   <si>
     <t>desfavoravel</t>
@@ -1798,7 +1798,7 @@
         <v>150</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="T2" s="2">
         <v>55.9</v>
@@ -1807,7 +1807,7 @@
         <v>23.8</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -1866,7 +1866,7 @@
         <v>150</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="T3" s="2">
         <v>74.09999999999999</v>
@@ -1875,7 +1875,7 @@
         <v>13.3</v>
       </c>
       <c r="V3" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -1934,7 +1934,7 @@
         <v>150</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T4" s="2">
         <v>66.40000000000001</v>
@@ -1943,7 +1943,7 @@
         <v>21.7</v>
       </c>
       <c r="V4" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:22">
@@ -2002,7 +2002,7 @@
         <v>150</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="T5" s="2">
         <v>72.7</v>
@@ -2011,7 +2011,7 @@
         <v>26.2</v>
       </c>
       <c r="V5" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:22">
@@ -2070,7 +2070,7 @@
         <v>150</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="T6" s="2">
         <v>67.3</v>
@@ -2079,7 +2079,7 @@
         <v>24.1</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -2138,7 +2138,7 @@
         <v>150</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="T7" s="2">
         <v>61.2</v>
@@ -2147,7 +2147,7 @@
         <v>31.6</v>
       </c>
       <c r="V7" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:22">
@@ -2206,7 +2206,7 @@
         <v>150</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="T8" s="2">
         <v>61.5</v>
@@ -2215,7 +2215,7 @@
         <v>12</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" spans="1:22">
@@ -2274,7 +2274,7 @@
         <v>150</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T9" s="2">
         <v>62.6</v>
@@ -2283,7 +2283,7 @@
         <v>38.9</v>
       </c>
       <c r="V9" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:22">
@@ -2342,7 +2342,7 @@
         <v>150</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="T10" s="2">
         <v>65.3</v>
@@ -2351,7 +2351,7 @@
         <v>30.6</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -2410,7 +2410,7 @@
         <v>151</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T11" s="2">
         <v>61.8</v>
@@ -2419,7 +2419,7 @@
         <v>26.8</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -2478,7 +2478,7 @@
         <v>150</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T12" s="2">
         <v>71.09999999999999</v>
@@ -2487,7 +2487,7 @@
         <v>9.4</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -2546,7 +2546,7 @@
         <v>150</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="T13" s="2">
         <v>66.3</v>
@@ -2555,7 +2555,7 @@
         <v>19.5</v>
       </c>
       <c r="V13" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="14" spans="1:22">
@@ -2614,7 +2614,7 @@
         <v>152</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="T14" s="2">
         <v>64.7</v>
@@ -2623,7 +2623,7 @@
         <v>47.6</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:22">
@@ -2682,7 +2682,7 @@
         <v>150</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T15" s="2">
         <v>65.7</v>
@@ -2691,7 +2691,7 @@
         <v>23.8</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16" spans="1:22">
@@ -2750,7 +2750,7 @@
         <v>150</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="T16" s="2">
         <v>75</v>
@@ -2759,7 +2759,7 @@
         <v>5.9</v>
       </c>
       <c r="V16" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="17" spans="1:22">
@@ -2818,7 +2818,7 @@
         <v>150</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="T17" s="2">
         <v>59.9</v>
@@ -2827,7 +2827,7 @@
         <v>23.3</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18" spans="1:22">
@@ -2886,7 +2886,7 @@
         <v>150</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="T18" s="2">
         <v>66.7</v>
@@ -2895,7 +2895,7 @@
         <v>21.3</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" spans="1:22">
@@ -2954,7 +2954,7 @@
         <v>152</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="T19" s="2">
         <v>61.9</v>
@@ -2963,7 +2963,7 @@
         <v>35.1</v>
       </c>
       <c r="V19" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -3022,7 +3022,7 @@
         <v>152</v>
       </c>
       <c r="S20" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="T20" s="2">
         <v>61.5</v>
@@ -3031,7 +3031,7 @@
         <v>28.2</v>
       </c>
       <c r="V20" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -3090,7 +3090,7 @@
         <v>150</v>
       </c>
       <c r="S21" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="T21" s="2">
         <v>64.59999999999999</v>
@@ -3099,7 +3099,7 @@
         <v>16.9</v>
       </c>
       <c r="V21" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" spans="1:22">
@@ -3158,7 +3158,7 @@
         <v>152</v>
       </c>
       <c r="S22" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="T22" s="2">
         <v>66.8</v>
@@ -3167,7 +3167,7 @@
         <v>28</v>
       </c>
       <c r="V22" s="2" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:22">
@@ -3226,7 +3226,7 @@
         <v>150</v>
       </c>
       <c r="S23" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T23" s="2">
         <v>64.2</v>
@@ -3235,7 +3235,7 @@
         <v>24.6</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="24" spans="1:22">
@@ -3294,7 +3294,7 @@
         <v>152</v>
       </c>
       <c r="S24" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T24" s="2">
         <v>65.3</v>
@@ -3303,7 +3303,7 @@
         <v>10.1</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="25" spans="1:22">
@@ -3362,7 +3362,7 @@
         <v>152</v>
       </c>
       <c r="S25" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="T25" s="2">
         <v>62.4</v>
@@ -3371,7 +3371,7 @@
         <v>23.3</v>
       </c>
       <c r="V25" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26" spans="1:22">
@@ -3430,7 +3430,7 @@
         <v>150</v>
       </c>
       <c r="S26" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="T26" s="2">
         <v>54.8</v>
@@ -3439,7 +3439,7 @@
         <v>31.8</v>
       </c>
       <c r="V26" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" spans="1:22">
@@ -3498,7 +3498,7 @@
         <v>150</v>
       </c>
       <c r="S27" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="T27" s="2">
         <v>60.3</v>
@@ -3507,7 +3507,7 @@
         <v>24.5</v>
       </c>
       <c r="V27" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:22">
@@ -3566,7 +3566,7 @@
         <v>152</v>
       </c>
       <c r="S28" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="T28" s="2">
         <v>66.3</v>
@@ -3575,7 +3575,7 @@
         <v>14.5</v>
       </c>
       <c r="V28" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:22">
@@ -3634,7 +3634,7 @@
         <v>151</v>
       </c>
       <c r="S29" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="T29" s="2">
         <v>66.7</v>
@@ -3643,7 +3643,7 @@
         <v>35.7</v>
       </c>
       <c r="V29" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="30" spans="1:22">
@@ -3702,7 +3702,7 @@
         <v>150</v>
       </c>
       <c r="S30" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="T30" s="2">
         <v>62.6</v>
@@ -3711,7 +3711,7 @@
         <v>5.6</v>
       </c>
       <c r="V30" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="1:22">
@@ -3770,7 +3770,7 @@
         <v>152</v>
       </c>
       <c r="S31" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="T31" s="2">
         <v>69.59999999999999</v>
@@ -3779,7 +3779,7 @@
         <v>20.6</v>
       </c>
       <c r="V31" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:22">
@@ -3838,7 +3838,7 @@
         <v>152</v>
       </c>
       <c r="S32" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="T32" s="2">
         <v>65.5</v>
@@ -3847,7 +3847,7 @@
         <v>25.8</v>
       </c>
       <c r="V32" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="33" spans="1:22">
@@ -3906,7 +3906,7 @@
         <v>150</v>
       </c>
       <c r="S33" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="T33" s="2">
         <v>57.1</v>
@@ -3915,7 +3915,7 @@
         <v>26.9</v>
       </c>
       <c r="V33" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:22">
@@ -3974,7 +3974,7 @@
         <v>150</v>
       </c>
       <c r="S34" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="T34" s="2">
         <v>58.2</v>
@@ -3983,7 +3983,7 @@
         <v>18.1</v>
       </c>
       <c r="V34" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="35" spans="1:22">
@@ -4042,7 +4042,7 @@
         <v>150</v>
       </c>
       <c r="S35" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="T35" s="2">
         <v>60.4</v>
@@ -4051,7 +4051,7 @@
         <v>7.8</v>
       </c>
       <c r="V35" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="36" spans="1:22">
@@ -4110,7 +4110,7 @@
         <v>150</v>
       </c>
       <c r="S36" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="T36" s="2">
         <v>67.7</v>
@@ -4119,7 +4119,7 @@
         <v>24.3</v>
       </c>
       <c r="V36" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="37" spans="1:22">
@@ -4178,7 +4178,7 @@
         <v>150</v>
       </c>
       <c r="S37" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="T37" s="2">
         <v>57.5</v>
@@ -4187,7 +4187,7 @@
         <v>30.4</v>
       </c>
       <c r="V37" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="38" spans="1:22">
@@ -4246,7 +4246,7 @@
         <v>152</v>
       </c>
       <c r="S38" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="T38" s="2">
         <v>64.8</v>
@@ -4255,7 +4255,7 @@
         <v>23.4</v>
       </c>
       <c r="V38" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="39" spans="1:22">
@@ -4314,7 +4314,7 @@
         <v>152</v>
       </c>
       <c r="S39" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="T39" s="2">
         <v>62.6</v>
@@ -4323,7 +4323,7 @@
         <v>20.9</v>
       </c>
       <c r="V39" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40" spans="1:22">
@@ -4382,7 +4382,7 @@
         <v>150</v>
       </c>
       <c r="S40" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="T40" s="2">
         <v>60.8</v>
@@ -4391,7 +4391,7 @@
         <v>14</v>
       </c>
       <c r="V40" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="41" spans="1:22">
@@ -4450,7 +4450,7 @@
         <v>150</v>
       </c>
       <c r="S41" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="T41" s="2">
         <v>66</v>
@@ -4459,7 +4459,7 @@
         <v>20.6</v>
       </c>
       <c r="V41" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="42" spans="1:22">
@@ -4518,7 +4518,7 @@
         <v>152</v>
       </c>
       <c r="S42" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="T42" s="2">
         <v>63</v>
@@ -4527,7 +4527,7 @@
         <v>26.3</v>
       </c>
       <c r="V42" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="43" spans="1:22">
@@ -4586,7 +4586,7 @@
         <v>150</v>
       </c>
       <c r="S43" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="T43" s="2">
         <v>68.09999999999999</v>
@@ -4595,7 +4595,7 @@
         <v>21</v>
       </c>
       <c r="V43" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="44" spans="1:22">
@@ -4654,7 +4654,7 @@
         <v>150</v>
       </c>
       <c r="S44" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="T44" s="2">
         <v>62.7</v>
@@ -4663,7 +4663,7 @@
         <v>21.7</v>
       </c>
       <c r="V44" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="45" spans="1:22">
@@ -4722,7 +4722,7 @@
         <v>150</v>
       </c>
       <c r="S45" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="T45" s="2">
         <v>58</v>
@@ -4731,7 +4731,7 @@
         <v>22.8</v>
       </c>
       <c r="V45" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="46" spans="1:22">
@@ -4790,7 +4790,7 @@
         <v>152</v>
       </c>
       <c r="S46" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="T46" s="2">
         <v>68.40000000000001</v>
@@ -4799,7 +4799,7 @@
         <v>21.8</v>
       </c>
       <c r="V46" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="47" spans="1:22">
@@ -4858,7 +4858,7 @@
         <v>152</v>
       </c>
       <c r="S47" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="T47" s="2">
         <v>67.40000000000001</v>
@@ -4867,7 +4867,7 @@
         <v>8.6</v>
       </c>
       <c r="V47" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:22">
@@ -4926,7 +4926,7 @@
         <v>153</v>
       </c>
       <c r="S48" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="T48" s="2">
         <v>64.3</v>
@@ -4935,7 +4935,7 @@
         <v>19.5</v>
       </c>
       <c r="V48" s="2" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="49" spans="1:22">
@@ -4994,7 +4994,7 @@
         <v>150</v>
       </c>
       <c r="S49" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="T49" s="2">
         <v>62.1</v>
@@ -5003,7 +5003,7 @@
         <v>20.3</v>
       </c>
       <c r="V49" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="50" spans="1:22">
@@ -5062,7 +5062,7 @@
         <v>152</v>
       </c>
       <c r="S50" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="T50" s="2">
         <v>61.3</v>
@@ -5071,7 +5071,7 @@
         <v>22.6</v>
       </c>
       <c r="V50" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="51" spans="1:22">
@@ -5130,7 +5130,7 @@
         <v>150</v>
       </c>
       <c r="S51" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="T51" s="5">
         <v>50</v>
@@ -5139,7 +5139,7 @@
         <v>41.2</v>
       </c>
       <c r="V51" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="52" spans="1:22">
@@ -5198,7 +5198,7 @@
         <v>153</v>
       </c>
       <c r="S52" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="T52" s="5">
         <v>71.40000000000001</v>
@@ -5266,7 +5266,7 @@
         <v>152</v>
       </c>
       <c r="S53" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T53" s="5">
         <v>64.40000000000001</v>
@@ -5275,7 +5275,7 @@
         <v>5.9</v>
       </c>
       <c r="V53" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:22">
@@ -5334,7 +5334,7 @@
         <v>152</v>
       </c>
       <c r="S54" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="T54" s="5">
         <v>60.5</v>
@@ -5343,7 +5343,7 @@
         <v>28.4</v>
       </c>
       <c r="V54" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="55" spans="1:22">
@@ -5402,7 +5402,7 @@
         <v>152</v>
       </c>
       <c r="S55" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="T55" s="5">
         <v>63.5</v>
@@ -5411,7 +5411,7 @@
         <v>10.9</v>
       </c>
       <c r="V55" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="56" spans="1:22">
@@ -5470,7 +5470,7 @@
         <v>153</v>
       </c>
       <c r="S56" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="T56" s="5">
         <v>66.7</v>
@@ -5535,10 +5535,10 @@
         <v>2088.813720703125</v>
       </c>
       <c r="R57" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="S57" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="T57" s="5">
         <v>69.09999999999999</v>
@@ -5547,7 +5547,7 @@
         <v>17</v>
       </c>
       <c r="V57" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="58" spans="1:22">
@@ -5606,7 +5606,7 @@
         <v>152</v>
       </c>
       <c r="S58" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="T58" s="5">
         <v>55.9</v>
@@ -5615,7 +5615,7 @@
         <v>32.5</v>
       </c>
       <c r="V58" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="59" spans="1:22">
@@ -5674,7 +5674,7 @@
         <v>150</v>
       </c>
       <c r="S59" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="T59" s="5">
         <v>55.6</v>
@@ -5683,7 +5683,7 @@
         <v>21</v>
       </c>
       <c r="V59" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="60" spans="1:22">
@@ -5742,7 +5742,7 @@
         <v>153</v>
       </c>
       <c r="S60" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="T60" s="5">
         <v>70.8</v>
@@ -5810,7 +5810,7 @@
         <v>152</v>
       </c>
       <c r="S61" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="T61" s="5">
         <v>68.7</v>
@@ -5819,7 +5819,7 @@
         <v>28.2</v>
       </c>
       <c r="V61" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="62" spans="1:22">
@@ -5878,7 +5878,7 @@
         <v>150</v>
       </c>
       <c r="S62" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="T62" s="5">
         <v>57.4</v>
@@ -5887,7 +5887,7 @@
         <v>25.2</v>
       </c>
       <c r="V62" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="63" spans="1:22">
@@ -5946,7 +5946,7 @@
         <v>153</v>
       </c>
       <c r="S63" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="T63" s="5">
         <v>62.1</v>
@@ -6014,7 +6014,7 @@
         <v>153</v>
       </c>
       <c r="S64" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="T64" s="5">
         <v>60</v>
@@ -6082,7 +6082,7 @@
         <v>153</v>
       </c>
       <c r="S65" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="T65" s="5">
         <v>68.3</v>
@@ -6091,7 +6091,7 @@
         <v>12.4</v>
       </c>
       <c r="V65" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="66" spans="1:22">
@@ -6150,7 +6150,7 @@
         <v>152</v>
       </c>
       <c r="S66" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="T66" s="5">
         <v>70.5</v>
@@ -6159,7 +6159,7 @@
         <v>13.1</v>
       </c>
       <c r="V66" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="67" spans="1:22">
@@ -6218,7 +6218,7 @@
         <v>153</v>
       </c>
       <c r="S67" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="T67" s="5">
         <v>66.7</v>
@@ -6227,7 +6227,7 @@
         <v>20.1</v>
       </c>
       <c r="V67" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="68" spans="1:22">
@@ -6286,7 +6286,7 @@
         <v>150</v>
       </c>
       <c r="S68" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="T68" s="5">
         <v>64.59999999999999</v>
@@ -6295,7 +6295,7 @@
         <v>36.3</v>
       </c>
       <c r="V68" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="69" spans="1:22">
@@ -6354,7 +6354,7 @@
         <v>152</v>
       </c>
       <c r="S69" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="T69" s="5">
         <v>51.6</v>
@@ -6363,7 +6363,7 @@
         <v>12.7</v>
       </c>
       <c r="V69" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="70" spans="1:22">
@@ -6422,7 +6422,7 @@
         <v>150</v>
       </c>
       <c r="S70" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="T70" s="5">
         <v>64.3</v>
@@ -6431,7 +6431,7 @@
         <v>20.9</v>
       </c>
       <c r="V70" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="71" spans="1:22">
@@ -6490,7 +6490,7 @@
         <v>153</v>
       </c>
       <c r="S71" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="T71" s="5">
         <v>60.3</v>
@@ -6558,7 +6558,7 @@
         <v>153</v>
       </c>
       <c r="S72" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="T72" s="5">
         <v>62.9</v>
@@ -6567,7 +6567,7 @@
         <v>17.4</v>
       </c>
       <c r="V72" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="73" spans="1:22">
@@ -6626,7 +6626,7 @@
         <v>152</v>
       </c>
       <c r="S73" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="T73" s="5">
         <v>65.3</v>
@@ -6635,7 +6635,7 @@
         <v>27.8</v>
       </c>
       <c r="V73" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="74" spans="1:22">
@@ -6694,7 +6694,7 @@
         <v>150</v>
       </c>
       <c r="S74" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="T74" s="5">
         <v>53.4</v>
@@ -6703,7 +6703,7 @@
         <v>22.8</v>
       </c>
       <c r="V74" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="75" spans="1:22">
@@ -6762,7 +6762,7 @@
         <v>151</v>
       </c>
       <c r="S75" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="T75" s="5">
         <v>62.8</v>
@@ -6771,7 +6771,7 @@
         <v>30.8</v>
       </c>
       <c r="V75" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="76" spans="1:22">
@@ -6830,7 +6830,7 @@
         <v>152</v>
       </c>
       <c r="S76" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="T76" s="5">
         <v>57.8</v>
@@ -6839,7 +6839,7 @@
         <v>7.9</v>
       </c>
       <c r="V76" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="77" spans="1:22">
@@ -6898,7 +6898,7 @@
         <v>153</v>
       </c>
       <c r="S77" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="T77" s="5">
         <v>57.7</v>
@@ -6907,7 +6907,7 @@
         <v>41</v>
       </c>
       <c r="V77" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="78" spans="1:22">
@@ -6966,7 +6966,7 @@
         <v>153</v>
       </c>
       <c r="S78" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="T78" s="5">
         <v>83.3</v>
@@ -7034,7 +7034,7 @@
         <v>153</v>
       </c>
       <c r="S79" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="T79" s="5">
         <v>64.3</v>
@@ -7043,7 +7043,7 @@
         <v>29.3</v>
       </c>
       <c r="V79" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="80" spans="1:22">
@@ -7102,7 +7102,7 @@
         <v>150</v>
       </c>
       <c r="S80" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="T80" s="5">
         <v>59</v>
@@ -7111,7 +7111,7 @@
         <v>24.2</v>
       </c>
       <c r="V80" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="81" spans="1:22">
@@ -7170,7 +7170,7 @@
         <v>150</v>
       </c>
       <c r="S81" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="T81" s="5">
         <v>48.4</v>
@@ -7179,7 +7179,7 @@
         <v>24.5</v>
       </c>
       <c r="V81" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="82" spans="1:22">
@@ -7238,7 +7238,7 @@
         <v>153</v>
       </c>
       <c r="S82" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="T82" s="5">
         <v>58.3</v>
@@ -7306,7 +7306,7 @@
         <v>152</v>
       </c>
       <c r="S83" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="T83" s="5">
         <v>69.09999999999999</v>
@@ -7315,7 +7315,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="V83" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="84" spans="1:22">
@@ -7374,7 +7374,7 @@
         <v>152</v>
       </c>
       <c r="S84" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="T84" s="5">
         <v>47.4</v>
@@ -7383,7 +7383,7 @@
         <v>18.2</v>
       </c>
       <c r="V84" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="85" spans="1:22">
@@ -7442,7 +7442,7 @@
         <v>153</v>
       </c>
       <c r="S85" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="T85" s="5">
         <v>66.40000000000001</v>
@@ -7510,7 +7510,7 @@
         <v>153</v>
       </c>
       <c r="S86" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="T86" s="5">
         <v>65.8</v>
@@ -7519,7 +7519,7 @@
         <v>34.5</v>
       </c>
       <c r="V86" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="87" spans="1:22">
@@ -7578,7 +7578,7 @@
         <v>152</v>
       </c>
       <c r="S87" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="T87" s="5">
         <v>51.6</v>
@@ -7587,7 +7587,7 @@
         <v>21.3</v>
       </c>
       <c r="V87" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="88" spans="1:22">
@@ -7646,7 +7646,7 @@
         <v>152</v>
       </c>
       <c r="S88" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="T88" s="5">
         <v>50</v>
@@ -7655,7 +7655,7 @@
         <v>7</v>
       </c>
       <c r="V88" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="89" spans="1:22">
@@ -7714,7 +7714,7 @@
         <v>153</v>
       </c>
       <c r="S89" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="T89" s="5">
         <v>65.5</v>
@@ -7723,7 +7723,7 @@
         <v>17.8</v>
       </c>
       <c r="V89" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="90" spans="1:22">
@@ -7782,7 +7782,7 @@
         <v>153</v>
       </c>
       <c r="S90" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="T90" s="5">
         <v>52.2</v>
@@ -7850,7 +7850,7 @@
         <v>152</v>
       </c>
       <c r="S91" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="T91" s="5">
         <v>55.9</v>
@@ -7859,7 +7859,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="V91" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="92" spans="1:22">
@@ -7918,7 +7918,7 @@
         <v>152</v>
       </c>
       <c r="S92" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="T92" s="5">
         <v>30.8</v>
@@ -7927,7 +7927,7 @@
         <v>20.3</v>
       </c>
       <c r="V92" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="93" spans="1:22">
@@ -7986,7 +7986,7 @@
         <v>152</v>
       </c>
       <c r="S93" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="T93" s="5">
         <v>63.4</v>
@@ -7995,7 +7995,7 @@
         <v>15.9</v>
       </c>
       <c r="V93" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="94" spans="1:22">
@@ -8054,7 +8054,7 @@
         <v>150</v>
       </c>
       <c r="S94" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="T94" s="5">
         <v>50</v>
@@ -8063,7 +8063,7 @@
         <v>19.5</v>
       </c>
       <c r="V94" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="95" spans="1:22">
@@ -8122,7 +8122,7 @@
         <v>153</v>
       </c>
       <c r="S95" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="T95" s="5">
         <v>54.2</v>
@@ -8131,7 +8131,7 @@
         <v>24</v>
       </c>
       <c r="V95" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="96" spans="1:22">
@@ -8190,7 +8190,7 @@
         <v>152</v>
       </c>
       <c r="S96" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="T96" s="5">
         <v>58.8</v>
@@ -8199,7 +8199,7 @@
         <v>22.6</v>
       </c>
       <c r="V96" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="97" spans="1:22">
@@ -8258,7 +8258,7 @@
         <v>153</v>
       </c>
       <c r="S97" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="T97" s="5">
         <v>66.2</v>
@@ -8267,7 +8267,7 @@
         <v>10.6</v>
       </c>
       <c r="V97" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="98" spans="1:22">
@@ -8326,7 +8326,7 @@
         <v>152</v>
       </c>
       <c r="S98" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="T98" s="5">
         <v>60</v>
@@ -8335,7 +8335,7 @@
         <v>50</v>
       </c>
       <c r="V98" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="99" spans="1:22">
@@ -8394,7 +8394,7 @@
         <v>153</v>
       </c>
       <c r="S99" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="T99" s="5">
         <v>69</v>
@@ -8403,7 +8403,7 @@
         <v>21.1</v>
       </c>
       <c r="V99" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="100" spans="1:22">
@@ -8462,7 +8462,7 @@
         <v>152</v>
       </c>
       <c r="S100" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="T100" s="5">
         <v>48.8</v>
@@ -8471,7 +8471,7 @@
         <v>17.6</v>
       </c>
       <c r="V100" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="101" spans="1:22">
@@ -8530,7 +8530,7 @@
         <v>153</v>
       </c>
       <c r="S101" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="T101" s="5">
         <v>33.3</v>
@@ -8598,7 +8598,7 @@
         <v>153</v>
       </c>
       <c r="S102" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="T102" s="5">
         <v>53.6</v>
@@ -8607,7 +8607,7 @@
         <v>7</v>
       </c>
       <c r="V102" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="103" spans="1:22">
@@ -8666,7 +8666,7 @@
         <v>153</v>
       </c>
       <c r="S103" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="T103" s="5">
         <v>64.3</v>
@@ -8734,7 +8734,7 @@
         <v>150</v>
       </c>
       <c r="S104" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T104" s="5">
         <v>49.1</v>
@@ -8743,7 +8743,7 @@
         <v>19.4</v>
       </c>
       <c r="V104" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="105" spans="1:22">
@@ -8802,7 +8802,7 @@
         <v>153</v>
       </c>
       <c r="S105" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T105" s="5">
         <v>62.8</v>
@@ -8811,7 +8811,7 @@
         <v>8.6</v>
       </c>
       <c r="V105" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="106" spans="1:22">
@@ -8870,7 +8870,7 @@
         <v>152</v>
       </c>
       <c r="S106" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="T106" s="5">
         <v>46.2</v>
@@ -8879,7 +8879,7 @@
         <v>21.1</v>
       </c>
       <c r="V106" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="107" spans="1:22">
@@ -8938,7 +8938,7 @@
         <v>152</v>
       </c>
       <c r="S107" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="T107" s="5">
         <v>46.2</v>
@@ -8947,7 +8947,7 @@
         <v>14</v>
       </c>
       <c r="V107" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="108" spans="1:22">
@@ -9006,7 +9006,7 @@
         <v>153</v>
       </c>
       <c r="S108" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="T108" s="5">
         <v>62.8</v>
@@ -9015,7 +9015,7 @@
         <v>10.7</v>
       </c>
       <c r="V108" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="109" spans="1:22">
@@ -9074,7 +9074,7 @@
         <v>152</v>
       </c>
       <c r="S109" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="T109" s="5">
         <v>40</v>
@@ -9083,7 +9083,7 @@
         <v>23.8</v>
       </c>
       <c r="V109" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="110" spans="1:22">
@@ -9142,7 +9142,7 @@
         <v>153</v>
       </c>
       <c r="S110" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="T110" s="5">
         <v>22.2</v>
@@ -9210,7 +9210,7 @@
         <v>152</v>
       </c>
       <c r="S111" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="T111" s="5">
         <v>48.7</v>
@@ -9219,7 +9219,7 @@
         <v>13.3</v>
       </c>
       <c r="V111" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="112" spans="1:22">
@@ -9278,7 +9278,7 @@
         <v>153</v>
       </c>
       <c r="S112" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="T112" s="5">
         <v>56</v>
@@ -9287,7 +9287,7 @@
         <v>5.7</v>
       </c>
       <c r="V112" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="113" spans="1:22">
@@ -9346,7 +9346,7 @@
         <v>153</v>
       </c>
       <c r="S113" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="T113" s="5">
         <v>53.8</v>
@@ -9355,7 +9355,7 @@
         <v>18.7</v>
       </c>
       <c r="V113" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="114" spans="1:22">
@@ -9414,7 +9414,7 @@
         <v>153</v>
       </c>
       <c r="S114" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="T114" s="5">
         <v>62.1</v>
@@ -9482,7 +9482,7 @@
         <v>153</v>
       </c>
       <c r="S115" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T115" s="5">
         <v>56.9</v>
@@ -9491,7 +9491,7 @@
         <v>16.6</v>
       </c>
       <c r="V115" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="116" spans="1:22">
@@ -9550,7 +9550,7 @@
         <v>153</v>
       </c>
       <c r="S116" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="T116" s="5">
         <v>58.1</v>
@@ -9618,7 +9618,7 @@
         <v>153</v>
       </c>
       <c r="S117" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="T117" s="5">
         <v>53.8</v>
@@ -9627,7 +9627,7 @@
         <v>32.8</v>
       </c>
       <c r="V117" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="118" spans="1:22">
@@ -9686,7 +9686,7 @@
         <v>152</v>
       </c>
       <c r="S118" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="T118" s="5">
         <v>51.7</v>
@@ -9695,7 +9695,7 @@
         <v>22.9</v>
       </c>
       <c r="V118" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="119" spans="1:22">
@@ -9754,7 +9754,7 @@
         <v>153</v>
       </c>
       <c r="S119" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="T119" s="5">
         <v>48.3</v>
@@ -9763,7 +9763,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="V119" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
     <row r="120" spans="1:22">
@@ -9822,7 +9822,7 @@
         <v>153</v>
       </c>
       <c r="S120" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="T120" s="5">
         <v>22.2</v>
@@ -9831,7 +9831,7 @@
         <v>20.6</v>
       </c>
       <c r="V120" s="5" t="s">
-        <v>154</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix entrada coherent with pivot: buy above pivot on breakout
When price is below pivot:
  entrada = pivot × 1.002 (buy on breakout confirmation)
  condicao = "COMPRAR a X se romper Pivot (Y)"

When price is above pivot:
  entrada = max(intraday_dip, pivot × 1.001) (never below pivot)
  condicao = "COMPRAR a X (acima do Pivot Y)"

When price is above R1:
  entrada = intraday_dip (desconto, momentum already confirmed)
  condicao = "COMPRAR a X (desconto intraday)"

All entrada values now >= pivot for breakout entries.

https://claude.ai/code/session_012uaj5aSEsJzsdD3tyDK1oP
</commit_message>
<xml_diff>
--- a/summary_latest.xlsx
+++ b/summary_latest.xlsx
@@ -682,157 +682,157 @@
     <t>muito cedo</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (65.27), limite em 64.32</t>
+    <t>COMPRAR a 65.34 (acima do Pivot 65.27). Stop em 62.17</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (29.17), limite em 28.94</t>
+    <t>COMPRAR a 29.20 (acima do Pivot 29.17). Stop em 28.09</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (48.21), limite em 46.85</t>
+    <t>COMPRAR a 48.26 (acima do Pivot 48.21). Stop em 44.77</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (9.58), limite em 9.41</t>
+    <t>COMPRAR a 9.59 (acima do Pivot 9.58). Stop em 9.02</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (8.63), limite em 8.54</t>
+    <t>COMPRAR a 8.64 (acima do Pivot 8.63). Stop em 8.37</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (165.72), limite em 165.07</t>
+    <t>COMPRAR a 165.89 (acima do Pivot 165.72). Stop em 161.77</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (45.02), limite em 44.45</t>
+    <t>COMPRAR a 45.07 (acima do Pivot 45.02). Stop em 42.91</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 63.76, limite em 61.80</t>
+    <t>COMPRAR a 63.89 se romper Pivot (63.76). Stop em 58.54</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (28.43), limite em 27.93</t>
+    <t>COMPRAR a 28.46 (acima do Pivot 28.43). Stop em 26.97</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 51.16, limite em 50.20</t>
+    <t>COMPRAR a 51.26 se romper Pivot (51.16). Stop em 48.78</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (14.20), limite em 14.00</t>
+    <t>COMPRAR a 14.21 (acima do Pivot 14.20). Stop em 13.62</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (94.66), limite em 94.20</t>
+    <t>COMPRAR a 94.76 (acima do Pivot 94.66). Stop em 92.32</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 57.25, limite em 56.08</t>
+    <t>COMPRAR a 57.37 se romper Pivot (57.25). Stop em 54.00</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (20.35), limite em 20.34</t>
+    <t>COMPRAR a 20.37 (acima do Pivot 20.35). Stop em 19.93</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (32.55), limite em 32.06</t>
+    <t>COMPRAR a 32.58 (acima do Pivot 32.55). Stop em 31.03</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (103.53), limite em 103.16</t>
+    <t>COMPRAR a 103.64 (acima do Pivot 103.53). Stop em 101.10</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (52.82), limite em 51.91</t>
+    <t>COMPRAR a 52.88 (acima do Pivot 52.82). Stop em 50.25</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 20.27, limite em 19.38</t>
+    <t>COMPRAR a 20.31 se romper Pivot (20.27). Stop em 18.39</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 47.32, limite em 46.47</t>
+    <t>COMPRAR a 47.42 se romper Pivot (47.32). Stop em 44.91</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (19.65), limite em 19.37</t>
+    <t>COMPRAR a 19.67 (acima do Pivot 19.65). Stop em 18.96</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (13.68), limite em 13.50</t>
+    <t>COMPRAR a 13.70 (acima do Pivot 13.68). Stop em 13.12</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 33.35, limite em 33.17</t>
+    <t>COMPRAR a 33.42 se romper Pivot (33.35). Stop em 32.51</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (41.40), limite em 41.09</t>
+    <t>COMPRAR a 41.44 (acima do Pivot 41.40). Stop em 40.19</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 157.47, limite em 154.14</t>
+    <t>COMPRAR a 157.78 se romper Pivot (157.47). Stop em 149.53</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (35.29), limite em 34.81</t>
+    <t>COMPRAR a 35.32 (acima do Pivot 35.29). Stop em 33.97</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 18.37, limite em 18.12</t>
+    <t>COMPRAR a 18.41 se romper Pivot (18.37). Stop em 17.72</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 18.13, limite em 17.65</t>
+    <t>COMPRAR a 18.16 se romper Pivot (18.13). Stop em 17.13</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 6.80, limite em 6.60</t>
+    <t>COMPRAR a 6.81 se romper Pivot (6.80). Stop em 6.37</t>
   </si>
   <si>
-    <t>COMPRAR: acima do Pivot (15.36), limite em 15.23</t>
+    <t>COMPRAR a 15.38 (acima do Pivot 15.36). Stop em 14.91</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 29.07, limite em 28.42</t>
+    <t>COMPRAR a 29.13 se romper Pivot (29.07). Stop em 27.71</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (23.53)</t>
+    <t>COMPRAR com cautela a 23.16. Cedo mas acima do Pivot (23.53)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (114.65)</t>
+    <t>COMPRAR com cautela a 114.27. Cedo mas acima do Pivot (114.65)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (46.77)</t>
+    <t>COMPRAR com cautela a 46.42. Cedo mas acima do Pivot (46.77)</t>
   </si>
   <si>
-    <t>CAUTELA: atrasado, considerar parcial. Pivot em 16.41</t>
+    <t>CAUTELA a 16.08: atrasado, considerar posicao parcial</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (31.27)</t>
+    <t>COMPRAR com cautela a 30.76. Cedo mas acima do Pivot (31.27)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (57.83)</t>
+    <t>COMPRAR com cautela a 56.71. Cedo mas acima do Pivot (57.83)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (16.02)</t>
+    <t>COMPRAR com cautela a 15.72. Cedo mas acima do Pivot (16.02)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (8.80)</t>
+    <t>COMPRAR com cautela a 8.70. Cedo mas acima do Pivot (8.80)</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 10.32, limite em 10.27</t>
+    <t>COMPRAR a 10.34 se romper Pivot (10.32). Stop em 10.06</t>
   </si>
   <si>
-    <t>CAUTELA: atrasado, considerar parcial. Pivot em 9.43</t>
+    <t>CAUTELA a 9.03: atrasado, considerar posicao parcial</t>
   </si>
   <si>
-    <t>AGUARDAR: cedo, comprar apenas se romper 9.45</t>
+    <t>AGUARDAR: comprar a 9.47 apenas se romper Pivot (9.45)</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 12.61, limite em 12.44</t>
+    <t>COMPRAR a 12.64 se romper Pivot (12.61). Stop em 12.11</t>
   </si>
   <si>
-    <t>COMPRAR no rompimento de 9.74, limite em 9.68</t>
+    <t>COMPRAR a 9.76 se romper Pivot (9.74). Stop em 9.49</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (108.80)</t>
+    <t>COMPRAR com cautela a 108.42. Cedo mas acima do Pivot (108.80)</t>
   </si>
   <si>
-    <t>AGUARDAR: cedo, comprar apenas se romper 21.05</t>
+    <t>AGUARDAR: comprar a 21.09 apenas se romper Pivot (21.05)</t>
   </si>
   <si>
-    <t>AGUARDAR: cedo, comprar apenas se romper 23.17</t>
+    <t>AGUARDAR: comprar a 23.22 apenas se romper Pivot (23.17)</t>
   </si>
   <si>
-    <t>AGUARDAR: cedo, comprar apenas se romper 8.88</t>
+    <t>AGUARDAR: comprar a 8.89 apenas se romper Pivot (8.88)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (17.65)</t>
+    <t>COMPRAR com cautela a 17.41. Cedo mas acima do Pivot (17.65)</t>
   </si>
   <si>
-    <t>COMPRAR com cautela: cedo mas acima do Pivot (25.94)</t>
+    <t>COMPRAR com cautela a 25.76. Cedo mas acima do Pivot (25.94)</t>
   </si>
   <si>
-    <t>AGUARDAR: cedo, comprar apenas se romper 32.85</t>
+    <t>AGUARDAR: comprar a 32.92 apenas se romper Pivot (32.85)</t>
   </si>
   <si>
-    <t>AGUARDAR: cedo, comprar apenas se romper 48.78</t>
+    <t>AGUARDAR: comprar a 48.88 apenas se romper Pivot (48.78)</t>
   </si>
   <si>
     <t>HOLD: acima do Pivot (27.56) mas sem sinal</t>
@@ -1765,7 +1765,7 @@
         <v>65.61000061035156</v>
       </c>
       <c r="H2" s="4">
-        <v>64.32489776611328</v>
+        <v>65.33860015869141</v>
       </c>
       <c r="I2" s="2">
         <v>67.14569854736328</v>
@@ -1833,7 +1833,7 @@
         <v>29.32999992370605</v>
       </c>
       <c r="H3" s="4">
-        <v>28.94280052185059</v>
+        <v>29.19589996337891</v>
       </c>
       <c r="I3" s="2">
         <v>30.02449989318848</v>
@@ -1901,7 +1901,7 @@
         <v>48.25</v>
       </c>
       <c r="H4" s="4">
-        <v>46.84519958496094</v>
+        <v>48.26150131225586</v>
       </c>
       <c r="I4" s="2">
         <v>49.52489852905273</v>
@@ -1969,7 +1969,7 @@
         <v>9.609999656677246</v>
       </c>
       <c r="H5" s="4">
-        <v>9.414799690246582</v>
+        <v>9.589599609375</v>
       </c>
       <c r="I5" s="2">
         <v>9.836600303649902</v>
@@ -2037,7 +2037,7 @@
         <v>8.630000114440918</v>
       </c>
       <c r="H6" s="4">
-        <v>8.540499687194824</v>
+        <v>8.635299682617188</v>
       </c>
       <c r="I6" s="2">
         <v>8.69890022277832</v>
@@ -2105,7 +2105,7 @@
         <v>166.0700073242188</v>
       </c>
       <c r="H7" s="4">
-        <v>165.0675964355469</v>
+        <v>165.8890075683594</v>
       </c>
       <c r="I7" s="2">
         <v>167.5576934814453</v>
@@ -2173,7 +2173,7 @@
         <v>45.36000061035156</v>
       </c>
       <c r="H8" s="4">
-        <v>44.45159912109375</v>
+        <v>45.06829833984375</v>
       </c>
       <c r="I8" s="2">
         <v>46.22019958496094</v>
@@ -2241,7 +2241,7 @@
         <v>63.27999877929688</v>
       </c>
       <c r="H9" s="4">
-        <v>61.80089950561523</v>
+        <v>63.88750076293945</v>
       </c>
       <c r="I9" s="2">
         <v>65.17839813232422</v>
@@ -2309,7 +2309,7 @@
         <v>28.47999954223633</v>
       </c>
       <c r="H10" s="4">
-        <v>27.92880058288574</v>
+        <v>28.45509910583496</v>
       </c>
       <c r="I10" s="2">
         <v>28.99760055541992</v>
@@ -2377,7 +2377,7 @@
         <v>51.06999969482422</v>
       </c>
       <c r="H11" s="4">
-        <v>50.19850158691406</v>
+        <v>51.25899887084961</v>
       </c>
       <c r="I11" s="2">
         <v>52.24760055541992</v>
@@ -2445,7 +2445,7 @@
         <v>14.27000045776367</v>
       </c>
       <c r="H12" s="4">
-        <v>14.00090026855469</v>
+        <v>14.21420001983643</v>
       </c>
       <c r="I12" s="2">
         <v>14.57870006561279</v>
@@ -2513,7 +2513,7 @@
         <v>94.69000244140625</v>
       </c>
       <c r="H13" s="4">
-        <v>94.20390319824219</v>
+        <v>94.75800323486328</v>
       </c>
       <c r="I13" s="2">
         <v>95.28060150146484</v>
@@ -2581,7 +2581,7 @@
         <v>57.20000076293945</v>
       </c>
       <c r="H14" s="4">
-        <v>56.08459854125977</v>
+        <v>57.36780166625977</v>
       </c>
       <c r="I14" s="2">
         <v>58.77700042724609</v>
@@ -2649,7 +2649,7 @@
         <v>20.44000053405762</v>
       </c>
       <c r="H15" s="4">
-        <v>20.33779907226562</v>
+        <v>20.37369918823242</v>
       </c>
       <c r="I15" s="2">
         <v>20.54080009460449</v>
@@ -2717,7 +2717,7 @@
         <v>32.61000061035156</v>
       </c>
       <c r="H16" s="4">
-        <v>32.06480026245117</v>
+        <v>32.57920074462891</v>
       </c>
       <c r="I16" s="2">
         <v>33.35850143432617</v>
@@ -2785,7 +2785,7 @@
         <v>103.6800003051758</v>
       </c>
       <c r="H17" s="4">
-        <v>103.1615982055664</v>
+        <v>103.6368026733398</v>
       </c>
       <c r="I17" s="2">
         <v>104.0804977416992</v>
@@ -2853,7 +2853,7 @@
         <v>52.86999893188477</v>
       </c>
       <c r="H18" s="4">
-        <v>51.90660095214844</v>
+        <v>52.8760986328125</v>
       </c>
       <c r="I18" s="2">
         <v>53.99990081787109</v>
@@ -2921,7 +2921,7 @@
         <v>19.8700008392334</v>
       </c>
       <c r="H19" s="4">
-        <v>19.38050079345703</v>
+        <v>20.31380081176758</v>
       </c>
       <c r="I19" s="2">
         <v>20.46610069274902</v>
@@ -2989,7 +2989,7 @@
         <v>47.13000106811523</v>
       </c>
       <c r="H20" s="4">
-        <v>46.46960067749023</v>
+        <v>47.41790008544922</v>
       </c>
       <c r="I20" s="2">
         <v>48.4900016784668</v>
@@ -3057,7 +3057,7 @@
         <v>19.67000007629395</v>
       </c>
       <c r="H21" s="4">
-        <v>19.36689949035645</v>
+        <v>19.66629981994629</v>
       </c>
       <c r="I21" s="2">
         <v>19.9871997833252</v>
@@ -3125,7 +3125,7 @@
         <v>13.76000022888184</v>
       </c>
       <c r="H22" s="4">
-        <v>13.5044002532959</v>
+        <v>13.69699954986572</v>
       </c>
       <c r="I22" s="2">
         <v>14.00380039215088</v>
@@ -3193,7 +3193,7 @@
         <v>33.34000015258789</v>
       </c>
       <c r="H23" s="4">
-        <v>33.17330169677734</v>
+        <v>33.41669845581055</v>
       </c>
       <c r="I23" s="2">
         <v>33.43999862670898</v>
@@ -3261,7 +3261,7 @@
         <v>41.68999862670898</v>
       </c>
       <c r="H24" s="4">
-        <v>41.08879852294922</v>
+        <v>41.44469833374023</v>
       </c>
       <c r="I24" s="2">
         <v>42.51459884643555</v>
@@ -3329,7 +3329,7 @@
         <v>156.8899993896484</v>
       </c>
       <c r="H25" s="4">
-        <v>154.1369018554688</v>
+        <v>157.7848968505859</v>
       </c>
       <c r="I25" s="2">
         <v>160.3861999511719</v>
@@ -3397,7 +3397,7 @@
         <v>35.36999893188477</v>
       </c>
       <c r="H26" s="4">
-        <v>34.81480026245117</v>
+        <v>35.32199859619141</v>
       </c>
       <c r="I26" s="2">
         <v>35.94929885864258</v>
@@ -3465,7 +3465,7 @@
         <v>18.36000061035156</v>
       </c>
       <c r="H27" s="4">
-        <v>18.1201000213623</v>
+        <v>18.40670013427734</v>
       </c>
       <c r="I27" s="2">
         <v>18.67490005493164</v>
@@ -3533,7 +3533,7 @@
         <v>17.88999938964844</v>
       </c>
       <c r="H28" s="4">
-        <v>17.64970016479492</v>
+        <v>18.16300010681152</v>
       </c>
       <c r="I28" s="2">
         <v>18.20730018615723</v>
@@ -3601,7 +3601,7 @@
         <v>6.769999980926514</v>
       </c>
       <c r="H29" s="4">
-        <v>6.603799819946289</v>
+        <v>6.810299873352051</v>
       </c>
       <c r="I29" s="2">
         <v>6.955599784851074</v>
@@ -3669,7 +3669,7 @@
         <v>15.43000030517578</v>
       </c>
       <c r="H30" s="4">
-        <v>15.22679996490479</v>
+        <v>15.37870025634766</v>
       </c>
       <c r="I30" s="2">
         <v>15.7101001739502</v>
@@ -3737,7 +3737,7 @@
         <v>28.89999961853027</v>
       </c>
       <c r="H31" s="4">
-        <v>28.42289924621582</v>
+        <v>29.12809944152832</v>
       </c>
       <c r="I31" s="2">
         <v>29.41729927062988</v>
@@ -4349,7 +4349,7 @@
         <v>10.31999969482422</v>
       </c>
       <c r="H40" s="4">
-        <v>10.26840019226074</v>
+        <v>10.34060001373291</v>
       </c>
       <c r="I40" s="2">
         <v>10.36450004577637</v>
@@ -4485,7 +4485,7 @@
         <v>9.170000076293945</v>
       </c>
       <c r="H42" s="4">
-        <v>8.9</v>
+        <v>9.46560001373291</v>
       </c>
       <c r="I42" s="2">
         <v>9.445099830627441</v>
@@ -4553,7 +4553,7 @@
         <v>12.60999965667725</v>
       </c>
       <c r="H43" s="4">
-        <v>12.43630027770996</v>
+        <v>12.63850021362305</v>
       </c>
       <c r="I43" s="2">
         <v>12.85079956054688</v>
@@ -4621,7 +4621,7 @@
         <v>9.729999542236328</v>
       </c>
       <c r="H44" s="4">
-        <v>9.681400299072266</v>
+        <v>9.762800216674805</v>
       </c>
       <c r="I44" s="2">
         <v>9.781100273132324</v>
@@ -4757,7 +4757,7 @@
         <v>20.82999992370605</v>
       </c>
       <c r="H46" s="4">
-        <v>20.48970031738281</v>
+        <v>21.08880043029785</v>
       </c>
       <c r="I46" s="2">
         <v>21.20680046081543</v>
@@ -4825,7 +4825,7 @@
         <v>22.89999961853027</v>
       </c>
       <c r="H47" s="4">
-        <v>22.38</v>
+        <v>23.21960067749023</v>
       </c>
       <c r="I47" s="2">
         <v>23.38540077209473</v>
@@ -4893,7 +4893,7 @@
         <v>8.810000419616699</v>
       </c>
       <c r="H48" s="4">
-        <v>8.545700073242188</v>
+        <v>8.894499778747559</v>
       </c>
       <c r="I48" s="2">
         <v>9.074299812316895</v>
@@ -5097,7 +5097,7 @@
         <v>32.81000137329102</v>
       </c>
       <c r="H51" s="4">
-        <v>32.22990036010742</v>
+        <v>32.91899871826172</v>
       </c>
       <c r="I51" s="2">
         <v>33.36069869995117</v>
@@ -5165,7 +5165,7 @@
         <v>48.54000091552734</v>
       </c>
       <c r="H52" s="4">
-        <v>47.59030151367188</v>
+        <v>48.87760162353516</v>
       </c>
       <c r="I52" s="2">
         <v>49.38449859619141</v>

</xml_diff>